<commit_message>
demo: exercise the new Office previews
Richer sample xlsx and docx so the readers have something to chew on,
and tile copy that no longer claims browsers can't preview them.

Loads the library from src/ rather than dist/, so the demo runs from a
clean checkout without a build step.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/assets/bill-of-materials.xlsx
+++ b/demo/assets/bill-of-materials.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bill of materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +29,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004D5BE3"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +50,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,40 +419,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Part no.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Unit cost</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>In stock</t>
         </is>
       </c>
     </row>
@@ -474,13 +468,14 @@
       <c r="C2" t="n">
         <v>12</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="D2" t="n">
         <v>184.5</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -491,19 +486,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Impeller, 140mm</t>
+          <t>Impeller 140mm "A" grade</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>12</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="D3" t="n">
         <v>96</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -520,13 +516,14 @@
       <c r="C4" t="n">
         <v>24</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="D4" t="n">
         <v>22.75</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -537,42 +534,84 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mounting bracket</t>
+          <t>Mounting bracket &lt;heavy&gt;</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>24</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+      <c r="D5" t="n">
         <v>41.2</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HCA-4400</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fastener pack M8</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>box</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>13.9</v>
+      <c r="E5" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D7" t="n">
+        <v>344.45</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46281.60416666666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Lead time (days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rajkot Castings</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gujarat Seals</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>